<commit_message>
Correct mobile broadband affordability scoring
</commit_message>
<xml_diff>
--- a/data/raw/Market/mobile-broadband-data-and-voice-high-consumption-basket-total.xlsx
+++ b/data/raw/Market/mobile-broadband-data-and-voice-high-consumption-basket-total.xlsx
@@ -25151,7 +25151,7 @@
         <v>2025</v>
       </c>
       <c r="E2">
-        <v>0.1927390505655999</v>
+        <v>0.8072609494344</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -25171,7 +25171,7 @@
         <v>2025</v>
       </c>
       <c r="E3">
-        <v>0.21724838054722997</v>
+        <v>0.78275161945277</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -25191,7 +25191,7 @@
         <v>2025</v>
       </c>
       <c r="E4">
-        <v>6.4778110799574587E-2</v>
+        <v>0.935221889200425</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -25211,7 +25211,7 @@
         <v>2025</v>
       </c>
       <c r="E5">
-        <v>0.25089432466402395</v>
+        <v>0.749105675335976</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -25231,7 +25231,7 @@
         <v>2025</v>
       </c>
       <c r="E6">
-        <v>0.15353379096973796</v>
+        <v>0.846466209030262</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -25251,7 +25251,7 @@
         <v>2025</v>
       </c>
       <c r="E7">
-        <v>0.13492216958329303</v>
+        <v>0.865077830416707</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -25271,7 +25271,7 @@
         <v>2025</v>
       </c>
       <c r="E8">
-        <v>0.24233781301363236</v>
+        <v>0.757662186986368</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
@@ -25291,7 +25291,7 @@
         <v>2025</v>
       </c>
       <c r="E9">
-        <v>9.0350962003287225E-2</v>
+        <v>0.909649037996713</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -25311,7 +25311,7 @@
         <v>2025</v>
       </c>
       <c r="E10">
-        <v>6.7001836991201782E-2</v>
+        <v>0.932998163008798</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
@@ -25331,7 +25331,7 @@
         <v>2025</v>
       </c>
       <c r="E11">
-        <v>0.16005994392342646</v>
+        <v>0.839940056076574</v>
       </c>
       <c r="F11" t="b">
         <v>1</v>
@@ -25351,7 +25351,7 @@
         <v>2025</v>
       </c>
       <c r="E12">
-        <v>0.24992748718940341</v>
+        <v>0.750072512810597</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -25371,7 +25371,7 @@
         <v>2025</v>
       </c>
       <c r="E13">
-        <v>0.13086145218988687</v>
+        <v>0.869138547810113</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -25391,7 +25391,7 @@
         <v>2025</v>
       </c>
       <c r="E14">
-        <v>5.0855651165039151E-2</v>
+        <v>0.949144348834961</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
@@ -25411,7 +25411,7 @@
         <v>2025</v>
       </c>
       <c r="E15">
-        <v>0.13414869960359663</v>
+        <v>0.865851300396403</v>
       </c>
       <c r="F15" t="b">
         <v>1</v>
@@ -25431,7 +25431,7 @@
         <v>2025</v>
       </c>
       <c r="E16">
-        <v>0.2605143575364981</v>
+        <v>0.739485642463502</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
@@ -25451,7 +25451,7 @@
         <v>2025</v>
       </c>
       <c r="E17">
-        <v>0.10528860098617421</v>
+        <v>0.894711399013826</v>
       </c>
       <c r="F17" t="b">
         <v>1</v>
@@ -25471,7 +25471,7 @@
         <v>2025</v>
       </c>
       <c r="E18">
-        <v>0.22271101227883591</v>
+        <v>0.777288987721164</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
@@ -25491,7 +25491,7 @@
         <v>2025</v>
       </c>
       <c r="E19">
-        <v>0.18679300009668373</v>
+        <v>0.813206999903316</v>
       </c>
       <c r="F19" t="b">
         <v>1</v>
@@ -25511,7 +25511,7 @@
         <v>2025</v>
       </c>
       <c r="E20">
-        <v>4.7084985014019143E-2</v>
+        <v>0.952915014985981</v>
       </c>
       <c r="F20" t="b">
         <v>1</v>
@@ -25531,7 +25531,7 @@
         <v>2025</v>
       </c>
       <c r="E21">
-        <v>9.271971381610751E-2</v>
+        <v>0.907280286183892</v>
       </c>
       <c r="F21" t="b">
         <v>1</v>
@@ -25551,7 +25551,7 @@
         <v>2025</v>
       </c>
       <c r="E22">
-        <v>0.24548003480614908</v>
+        <v>0.754519965193851</v>
       </c>
       <c r="F22" t="b">
         <v>1</v>
@@ -25571,7 +25571,7 @@
         <v>2025</v>
       </c>
       <c r="E23">
-        <v>0.19288407618679299</v>
+        <v>0.807115923813207</v>
       </c>
       <c r="F23" t="b">
         <v>1</v>
@@ -25591,7 +25591,7 @@
         <v>2025</v>
       </c>
       <c r="E24">
-        <v>0.14570240742531179</v>
+        <v>0.854297592574688</v>
       </c>
       <c r="F24" t="b">
         <v>1</v>
@@ -25611,7 +25611,7 @@
         <v>2025</v>
       </c>
       <c r="E25">
-        <v>9.6973798704437772E-2</v>
+        <v>0.903026201295562</v>
       </c>
       <c r="F25" t="b">
         <v>1</v>
@@ -25631,7 +25631,7 @@
         <v>2025</v>
       </c>
       <c r="E26">
-        <v>0.1569660640046408</v>
+        <v>0.843033935995359</v>
       </c>
       <c r="F26" t="b">
         <v>1</v>
@@ -25651,7 +25651,7 @@
         <v>2025</v>
       </c>
       <c r="E27">
-        <v>0.38625157111089625</v>
+        <v>0.613748428889104</v>
       </c>
       <c r="F27" t="b">
         <v>1</v>
@@ -25671,7 +25671,7 @@
         <v>2025</v>
       </c>
       <c r="E28">
-        <v>0.34569273905056558</v>
+        <v>0.654307260949434</v>
       </c>
       <c r="F28" t="b">
         <v>1</v>
@@ -25691,7 +25691,7 @@
         <v>2025</v>
       </c>
       <c r="E29">
-        <v>5.5061394179638401E-2</v>
+        <v>0.944938605820362</v>
       </c>
       <c r="F29" t="b">
         <v>1</v>
@@ -25711,7 +25711,7 @@
         <v>2025</v>
       </c>
       <c r="E30">
-        <v>0.25331141835057525</v>
+        <v>0.746688581649425</v>
       </c>
       <c r="F30" t="b">
         <v>1</v>
@@ -25731,7 +25731,7 @@
         <v>2025</v>
       </c>
       <c r="E31">
-        <v>0.15981823455477132</v>
+        <v>0.840181765445229</v>
       </c>
       <c r="F31" t="b">
         <v>1</v>
@@ -25751,7 +25751,7 @@
         <v>2025</v>
       </c>
       <c r="E32">
-        <v>0.13497051145702404</v>
+        <v>0.865029488542976</v>
       </c>
       <c r="F32" t="b">
         <v>1</v>
@@ -25771,7 +25771,7 @@
         <v>2025</v>
       </c>
       <c r="E33">
-        <v>0.22246930291018077</v>
+        <v>0.777530697089819</v>
       </c>
       <c r="F33" t="b">
         <v>1</v>
@@ -25791,7 +25791,7 @@
         <v>2025</v>
       </c>
       <c r="E34">
-        <v>0.28178478197814943</v>
+        <v>0.718215218021851</v>
       </c>
       <c r="F34" t="b">
         <v>1</v>
@@ -25811,7 +25811,7 @@
         <v>2025</v>
       </c>
       <c r="E35">
-        <v>0.13182828966450738</v>
+        <v>0.868171710335493</v>
       </c>
       <c r="F35" t="b">
         <v>1</v>
@@ -25831,7 +25831,7 @@
         <v>2025</v>
       </c>
       <c r="E36">
-        <v>0.21410615875471331</v>
+        <v>0.785893841245287</v>
       </c>
       <c r="F36" t="b">
         <v>1</v>
@@ -25851,7 +25851,7 @@
         <v>2025</v>
       </c>
       <c r="E37">
-        <v>5.7575171613651742E-2</v>
+        <v>0.942424828386348</v>
       </c>
       <c r="F37" t="b">
         <v>1</v>
@@ -25871,7 +25871,7 @@
         <v>2025</v>
       </c>
       <c r="E38">
-        <v>6.8258725708208456E-2</v>
+        <v>0.931741274291792</v>
       </c>
       <c r="F38" t="b">
         <v>1</v>
@@ -25891,7 +25891,7 @@
         <v>2025</v>
       </c>
       <c r="E39">
-        <v>0.10267813980469881</v>
+        <v>0.897321860195301</v>
       </c>
       <c r="F39" t="b">
         <v>1</v>
@@ -25911,7 +25911,7 @@
         <v>2025</v>
       </c>
       <c r="E40">
-        <v>0.27376003093879914</v>
+        <v>0.726239969061201</v>
       </c>
       <c r="F40" t="b">
         <v>1</v>
@@ -25931,7 +25931,7 @@
         <v>2025</v>
       </c>
       <c r="E41">
-        <v>0.1952044861258822</v>
+        <v>0.804795513874118</v>
       </c>
       <c r="F41" t="b">
         <v>1</v>
@@ -25951,7 +25951,7 @@
         <v>2025</v>
       </c>
       <c r="E42">
-        <v>0.19061200812143478</v>
+        <v>0.809387991878565</v>
       </c>
       <c r="F42" t="b">
         <v>1</v>
@@ -25971,7 +25971,7 @@
         <v>2025</v>
       </c>
       <c r="E43">
-        <v>0.13400367398240354</v>
+        <v>0.865996326017596</v>
       </c>
       <c r="F43" t="b">
         <v>1</v>
@@ -25991,7 +25991,7 @@
         <v>2025</v>
       </c>
       <c r="E44">
-        <v>9.3928260659383145E-2</v>
+        <v>0.906071739340617</v>
       </c>
       <c r="F44" t="b">
         <v>1</v>
@@ -26011,7 +26011,7 @@
         <v>2025</v>
       </c>
       <c r="E45">
-        <v>0.10098617422411291</v>
+        <v>0.899013825775887</v>
       </c>
       <c r="F45" t="b">
         <v>1</v>
@@ -26031,7 +26031,7 @@
         <v>2025</v>
       </c>
       <c r="E46">
-        <v>6.3182828966450735E-2</v>
+        <v>0.936817171033549</v>
       </c>
       <c r="F46" t="b">
         <v>1</v>
@@ -26051,7 +26051,7 @@
         <v>2025</v>
       </c>
       <c r="E47">
-        <v>8.1939475974088752E-2</v>
+        <v>0.918060524025911</v>
       </c>
       <c r="F47" t="b">
         <v>1</v>
@@ -26071,7 +26071,7 @@
         <v>2025</v>
       </c>
       <c r="E48">
-        <v>0.27815914144832249</v>
+        <v>0.721840858551678</v>
       </c>
       <c r="F48" t="b">
         <v>1</v>
@@ -26091,7 +26091,7 @@
         <v>2025</v>
       </c>
       <c r="E49">
-        <v>0.3320119887846853</v>
+        <v>0.667988011215315</v>
       </c>
       <c r="F49" t="b">
         <v>1</v>
@@ -26111,7 +26111,7 @@
         <v>2025</v>
       </c>
       <c r="E50">
-        <v>0.40500821811853427</v>
+        <v>0.594991781881466</v>
       </c>
       <c r="F50" t="b">
         <v>1</v>
@@ -26131,7 +26131,7 @@
         <v>2025</v>
       </c>
       <c r="E51">
-        <v>7.7685391085758476E-2</v>
+        <v>0.922314608914242</v>
       </c>
       <c r="F51" t="b">
         <v>1</v>
@@ -26151,7 +26151,7 @@
         <v>2025</v>
       </c>
       <c r="E52">
-        <v>0.15793290147926134</v>
+        <v>0.842067098520739</v>
       </c>
       <c r="F52" t="b">
         <v>1</v>
@@ -26171,7 +26171,7 @@
         <v>2025</v>
       </c>
       <c r="E53">
-        <v>6.6228367011505362E-2</v>
+        <v>0.933771632988495</v>
       </c>
       <c r="F53" t="b">
         <v>1</v>
@@ -26191,7 +26191,7 @@
         <v>2025</v>
       </c>
       <c r="E54">
-        <v>0.26443004930871117</v>
+        <v>0.735569950691289</v>
       </c>
       <c r="F54" t="b">
         <v>1</v>
@@ -26211,7 +26211,7 @@
         <v>2025</v>
       </c>
       <c r="E55">
-        <v>0.34076186793000096</v>
+        <v>0.659238132069999</v>
       </c>
       <c r="F55" t="b">
         <v>1</v>
@@ -26231,7 +26231,7 @@
         <v>2025</v>
       </c>
       <c r="E56">
-        <v>0.12153147055979888</v>
+        <v>0.878468529440201</v>
       </c>
       <c r="F56" t="b">
         <v>1</v>
@@ -26251,7 +26251,7 @@
         <v>2025</v>
       </c>
       <c r="E57">
-        <v>0.27777240645847434</v>
+        <v>0.722227593541526</v>
       </c>
       <c r="F57" t="b">
         <v>1</v>
@@ -26271,7 +26271,7 @@
         <v>2025</v>
       </c>
       <c r="E58">
-        <v>0.11389345451029681</v>
+        <v>0.886106545489703</v>
       </c>
       <c r="F58" t="b">
         <v>1</v>
@@ -26291,7 +26291,7 @@
         <v>2025</v>
       </c>
       <c r="E59">
-        <v>0.1249154017209707</v>
+        <v>0.875084598279029</v>
       </c>
       <c r="F59" t="b">
         <v>1</v>
@@ -26311,7 +26311,7 @@
         <v>2025</v>
       </c>
       <c r="E60">
-        <v>0.12622063231170838</v>
+        <v>0.873779367688292</v>
       </c>
       <c r="F60" t="b">
         <v>1</v>
@@ -26331,7 +26331,7 @@
         <v>2025</v>
       </c>
       <c r="E61">
-        <v>8.7305423958232611E-2</v>
+        <v>0.912694576041767</v>
       </c>
       <c r="F61" t="b">
         <v>1</v>
@@ -26351,7 +26351,7 @@
         <v>2025</v>
       </c>
       <c r="E62">
-        <v>6.4826452673305612E-2</v>
+        <v>0.935173547326694</v>
       </c>
       <c r="F62" t="b">
         <v>1</v>
@@ -26371,7 +26371,7 @@
         <v>2025</v>
       </c>
       <c r="E63">
-        <v>5.2789326114280187E-2</v>
+        <v>0.94721067388572</v>
       </c>
       <c r="F63" t="b">
         <v>1</v>
@@ -26391,7 +26391,7 @@
         <v>2025</v>
       </c>
       <c r="E64">
-        <v>0.14739437300589769</v>
+        <v>0.852605626994102</v>
       </c>
       <c r="F64" t="b">
         <v>1</v>
@@ -26411,7 +26411,7 @@
         <v>2025</v>
       </c>
       <c r="E65">
-        <v>0.4973895388185246</v>
+        <v>0.502610461181475</v>
       </c>
       <c r="F65" t="b">
         <v>1</v>
@@ -26431,7 +26431,7 @@
         <v>2025</v>
       </c>
       <c r="E66">
-        <v>0.30387701827322827</v>
+        <v>0.696122981726772</v>
       </c>
       <c r="F66" t="b">
         <v>1</v>
@@ -26451,7 +26451,7 @@
         <v>2025</v>
       </c>
       <c r="E67">
-        <v>6.4681427052112536E-2</v>
+        <v>0.935318572947887</v>
       </c>
       <c r="F67" t="b">
         <v>1</v>
@@ -26471,7 +26471,7 @@
         <v>2025</v>
       </c>
       <c r="E68">
-        <v>0.11664894131296528</v>
+        <v>0.883351058687035</v>
       </c>
       <c r="F68" t="b">
         <v>1</v>
@@ -26491,7 +26491,7 @@
         <v>2025</v>
       </c>
       <c r="E69">
-        <v>0.1972348448225853</v>
+        <v>0.802765155177415</v>
       </c>
       <c r="F69" t="b">
         <v>1</v>
@@ -26511,7 +26511,7 @@
         <v>2025</v>
       </c>
       <c r="E70">
-        <v>0.17006671178574881</v>
+        <v>0.829933288214251</v>
       </c>
       <c r="F70" t="b">
         <v>1</v>
@@ -26531,7 +26531,7 @@
         <v>2025</v>
       </c>
       <c r="E71">
-        <v>6.8210383834477431E-2</v>
+        <v>0.931789616165523</v>
       </c>
       <c r="F71" t="b">
         <v>1</v>
@@ -26551,7 +26551,7 @@
         <v>2025</v>
       </c>
       <c r="E72">
-        <v>9.6635405588320594E-2</v>
+        <v>0.903364594411679</v>
       </c>
       <c r="F72" t="b">
         <v>1</v>
@@ -26571,7 +26571,7 @@
         <v>2025</v>
       </c>
       <c r="E73">
-        <v>0.10654548970318088</v>
+        <v>0.893454510296819</v>
       </c>
       <c r="F73" t="b">
         <v>1</v>
@@ -26591,7 +26591,7 @@
         <v>2025</v>
       </c>
       <c r="E74">
-        <v>0.18215218021850527</v>
+        <v>0.817847819781495</v>
       </c>
       <c r="F74" t="b">
         <v>1</v>
@@ -26611,7 +26611,7 @@
         <v>2025</v>
       </c>
       <c r="E75">
-        <v>0.16030165329208157</v>
+        <v>0.839698346707918</v>
       </c>
       <c r="F75" t="b">
         <v>1</v>
@@ -26631,7 +26631,7 @@
         <v>2025</v>
       </c>
       <c r="E76">
-        <v>0.20119887846852941</v>
+        <v>0.798801121531471</v>
       </c>
       <c r="F76" t="b">
         <v>1</v>
@@ -26651,7 +26651,7 @@
         <v>2025</v>
       </c>
       <c r="E77">
-        <v>0.15788455960553027</v>
+        <v>0.84211544039447</v>
       </c>
       <c r="F77" t="b">
         <v>1</v>
@@ -26671,7 +26671,7 @@
         <v>2025</v>
       </c>
       <c r="E78">
-        <v>0.1195011118630958</v>
+        <v>0.880498888136904</v>
       </c>
       <c r="F78" t="b">
         <v>1</v>
@@ -26691,7 +26691,7 @@
         <v>2025</v>
       </c>
       <c r="E79">
-        <v>0.33994005607657352</v>
+        <v>0.660059943923426</v>
       </c>
       <c r="F79" t="b">
         <v>1</v>
@@ -26711,7 +26711,7 @@
         <v>2025</v>
       </c>
       <c r="E80">
-        <v>0.32587257082084503</v>
+        <v>0.674127429179155</v>
       </c>
       <c r="F80" t="b">
         <v>1</v>
@@ -26731,7 +26731,7 @@
         <v>2025</v>
       </c>
       <c r="E81">
-        <v>0.1595765251861162</v>
+        <v>0.840423474813884</v>
       </c>
       <c r="F81" t="b">
         <v>1</v>
@@ -26751,7 +26751,7 @@
         <v>2025</v>
       </c>
       <c r="E82">
-        <v>0.14700763801604949</v>
+        <v>0.852992361983951</v>
       </c>
       <c r="F82" t="b">
         <v>1</v>
@@ -26771,7 +26771,7 @@
         <v>2025</v>
       </c>
       <c r="E83">
-        <v>0.16871313932128007</v>
+        <v>0.83128686067872</v>
       </c>
       <c r="F83" t="b">
         <v>1</v>
@@ -26791,7 +26791,7 @@
         <v>2025</v>
       </c>
       <c r="E84">
-        <v>0.29169486609300971</v>
+        <v>0.70830513390699</v>
       </c>
       <c r="F84" t="b">
         <v>1</v>
@@ -26811,7 +26811,7 @@
         <v>2025</v>
       </c>
       <c r="E85">
-        <v>3.1808952915014982E-2</v>
+        <v>0.968191047084985</v>
       </c>
       <c r="F85" t="b">
         <v>1</v>
@@ -26831,7 +26831,7 @@
         <v>2025</v>
       </c>
       <c r="E86">
-        <v>0.25978922943053273</v>
+        <v>0.740210770569467</v>
       </c>
       <c r="F86" t="b">
         <v>1</v>
@@ -26851,7 +26851,7 @@
         <v>2025</v>
       </c>
       <c r="E87">
-        <v>7.5606690515324371E-2</v>
+        <v>0.924393309484676</v>
       </c>
       <c r="F87" t="b">
         <v>1</v>
@@ -26871,7 +26871,7 @@
         <v>2025</v>
       </c>
       <c r="E88">
-        <v>2.1415450062844437E-2</v>
+        <v>0.978584549937156</v>
       </c>
       <c r="F88" t="b">
         <v>1</v>
@@ -26891,7 +26891,7 @@
         <v>2025</v>
       </c>
       <c r="E89">
-        <v>0.20472783525089433</v>
+        <v>0.795272164749106</v>
       </c>
       <c r="F89" t="b">
         <v>1</v>
@@ -26911,7 +26911,7 @@
         <v>2025</v>
       </c>
       <c r="E90">
-        <v>7.2657836217731794E-2</v>
+        <v>0.927342163782268</v>
       </c>
       <c r="F90" t="b">
         <v>1</v>
@@ -26931,7 +26931,7 @@
         <v>2025</v>
       </c>
       <c r="E91">
-        <v>5.9992265300203032E-2</v>
+        <v>0.940007734699797</v>
       </c>
       <c r="F91" t="b">
         <v>1</v>
@@ -26951,7 +26951,7 @@
         <v>2025</v>
       </c>
       <c r="E92">
-        <v>0.10461181475393984</v>
+        <v>0.89538818524606</v>
       </c>
       <c r="F92" t="b">
         <v>1</v>
@@ -26971,7 +26971,7 @@
         <v>2025</v>
       </c>
       <c r="E93">
-        <v>1.822488639659673E-2</v>
+        <v>0.981775113603403</v>
       </c>
       <c r="F93" t="b">
         <v>1</v>
@@ -26991,7 +26991,7 @@
         <v>2025</v>
       </c>
       <c r="E94">
-        <v>0.12878275161945274</v>
+        <v>0.871217248380547</v>
       </c>
       <c r="F94" t="b">
         <v>1</v>
@@ -27011,7 +27011,7 @@
         <v>2025</v>
       </c>
       <c r="E95">
-        <v>8.3293048438557463E-2</v>
+        <v>0.916706951561443</v>
       </c>
       <c r="F95" t="b">
         <v>1</v>
@@ -27031,7 +27031,7 @@
         <v>2025</v>
       </c>
       <c r="E96">
-        <v>5.8251957845886104E-2</v>
+        <v>0.941748042154114</v>
       </c>
       <c r="F96" t="b">
         <v>1</v>
@@ -27051,7 +27051,7 @@
         <v>2025</v>
       </c>
       <c r="E97">
-        <v>0.11104128396016628</v>
+        <v>0.888958716039834</v>
       </c>
       <c r="F97" t="b">
         <v>1</v>
@@ -27071,7 +27071,7 @@
         <v>2025</v>
       </c>
       <c r="E98">
-        <v>0.25340810209803732</v>
+        <v>0.746591897901963</v>
       </c>
       <c r="F98" t="b">
         <v>1</v>
@@ -27091,7 +27091,7 @@
         <v>2025</v>
       </c>
       <c r="E99">
-        <v>0.16716619936188726</v>
+        <v>0.832833800638113</v>
       </c>
       <c r="F99" t="b">
         <v>1</v>
@@ -27111,7 +27111,7 @@
         <v>2025</v>
       </c>
       <c r="E100">
-        <v>0.14454220245576718</v>
+        <v>0.855457797544233</v>
       </c>
       <c r="F100" t="b">
         <v>1</v>
@@ -27131,7 +27131,7 @@
         <v>2025</v>
       </c>
       <c r="E101">
-        <v>0.1636855844532534</v>
+        <v>0.836314415546747</v>
       </c>
       <c r="F101" t="b">
         <v>1</v>
@@ -27151,7 +27151,7 @@
         <v>2025</v>
       </c>
       <c r="E102">
-        <v>0.1084308227786909</v>
+        <v>0.891569177221309</v>
       </c>
       <c r="F102" t="b">
         <v>1</v>
@@ -27171,7 +27171,7 @@
         <v>2025</v>
       </c>
       <c r="E103">
-        <v>4.3797737600309389E-2</v>
+        <v>0.956202262399691</v>
       </c>
       <c r="F103" t="b">
         <v>1</v>
@@ -27191,7 +27191,7 @@
         <v>2025</v>
       </c>
       <c r="E104">
-        <v>5.1000676786232234E-2</v>
+        <v>0.948999323213768</v>
       </c>
       <c r="F104" t="b">
         <v>1</v>
@@ -27211,7 +27211,7 @@
         <v>2025</v>
       </c>
       <c r="E105">
-        <v>0.23890553997872957</v>
+        <v>0.76109446002127</v>
       </c>
       <c r="F105" t="b">
         <v>1</v>
@@ -27231,7 +27231,7 @@
         <v>2025</v>
       </c>
       <c r="E106">
-        <v>0.22478971284927002</v>
+        <v>0.77521028715073</v>
       </c>
       <c r="F106" t="b">
         <v>1</v>
@@ -27251,7 +27251,7 @@
         <v>2025</v>
       </c>
       <c r="E107">
-        <v>0.13946630571400945</v>
+        <v>0.860533694285991</v>
       </c>
       <c r="F107" t="b">
         <v>1</v>
@@ -27271,7 +27271,7 @@
         <v>2025</v>
       </c>
       <c r="E108">
-        <v>7.2947887460117947E-2</v>
+        <v>0.927052112539882</v>
       </c>
       <c r="F108" t="b">
         <v>1</v>
@@ -27291,7 +27291,7 @@
         <v>2025</v>
       </c>
       <c r="E109">
-        <v>0.16784298559412161</v>
+        <v>0.832157014405878</v>
       </c>
       <c r="F109" t="b">
         <v>1</v>
@@ -27311,7 +27311,7 @@
         <v>2025</v>
       </c>
       <c r="E110">
-        <v>8.0730929130813103E-2</v>
+        <v>0.919269070869187</v>
       </c>
       <c r="F110" t="b">
         <v>1</v>
@@ -27331,7 +27331,7 @@
         <v>2025</v>
       </c>
       <c r="E111">
-        <v>0.11998453060040606</v>
+        <v>0.880015469399594</v>
       </c>
       <c r="F111" t="b">
         <v>1</v>
@@ -27351,7 +27351,7 @@
         <v>2025</v>
       </c>
       <c r="E112">
-        <v>9.9970994875761374E-2</v>
+        <v>0.900029005124239</v>
       </c>
       <c r="F112" t="b">
         <v>1</v>
@@ -27371,7 +27371,7 @@
         <v>2025</v>
       </c>
       <c r="E113">
-        <v>5.1387411776080444E-2</v>
+        <v>0.94861258822392</v>
       </c>
       <c r="F113" t="b">
         <v>1</v>
@@ -27391,7 +27391,7 @@
         <v>2025</v>
       </c>
       <c r="E114">
-        <v>0.40254278255825199</v>
+        <v>0.597457217441748</v>
       </c>
       <c r="F114" t="b">
         <v>1</v>
@@ -27411,7 +27411,7 @@
         <v>2025</v>
       </c>
       <c r="E115">
-        <v>0.10654548970318088</v>
+        <v>0.893454510296819</v>
       </c>
       <c r="F115" t="b">
         <v>1</v>
@@ -27431,7 +27431,7 @@
         <v>2025</v>
       </c>
       <c r="E116">
-        <v>3.8915208353475783E-2</v>
+        <v>0.961084791646524</v>
       </c>
       <c r="F116" t="b">
         <v>1</v>
@@ -27451,7 +27451,7 @@
         <v>2025</v>
       </c>
       <c r="E117">
-        <v>0.18108865899642268</v>
+        <v>0.818911341003577</v>
       </c>
       <c r="F117" t="b">
         <v>1</v>
@@ -27471,7 +27471,7 @@
         <v>2025</v>
       </c>
       <c r="E118">
-        <v>5.7236778497534557E-2</v>
+        <v>0.942763221502465</v>
       </c>
       <c r="F118" t="b">
         <v>1</v>
@@ -27491,7 +27491,7 @@
         <v>2025</v>
       </c>
       <c r="E119">
-        <v>5.9557188436623804E-2</v>
+        <v>0.940442811563376</v>
       </c>
       <c r="F119" t="b">
         <v>1</v>
@@ -27511,7 +27511,7 @@
         <v>2025</v>
       </c>
       <c r="E120">
-        <v>0.14135163878951945</v>
+        <v>0.85864836121048</v>
       </c>
       <c r="F120" t="b">
         <v>1</v>
@@ -27531,7 +27531,7 @@
         <v>2025</v>
       </c>
       <c r="E121">
-        <v>8.633858648361209E-2</v>
+        <v>0.913661413516388</v>
       </c>
       <c r="F121" t="b">
         <v>1</v>
@@ -27551,7 +27551,7 @@
         <v>2025</v>
       </c>
       <c r="E122">
-        <v>8.3293048438557463E-2</v>
+        <v>0.916706951561443</v>
       </c>
       <c r="F122" t="b">
         <v>1</v>
@@ -27571,7 +27571,7 @@
         <v>2025</v>
       </c>
       <c r="E123">
-        <v>0.25374649521415449</v>
+        <v>0.746253504785846</v>
       </c>
       <c r="F123" t="b">
         <v>1</v>
@@ -27591,7 +27591,7 @@
         <v>2025</v>
       </c>
       <c r="E124">
-        <v>3.9978729575558342E-2</v>
+        <v>0.960021270424442</v>
       </c>
       <c r="F124" t="b">
         <v>1</v>
@@ -27611,7 +27611,7 @@
         <v>2025</v>
       </c>
       <c r="E125">
-        <v>0.15155177414676591</v>
+        <v>0.848448225853234</v>
       </c>
       <c r="F125" t="b">
         <v>1</v>
@@ -27631,7 +27631,7 @@
         <v>2025</v>
       </c>
       <c r="E126">
-        <v>0.17620612974958907</v>
+        <v>0.823793870250411</v>
       </c>
       <c r="F126" t="b">
         <v>1</v>
@@ -27651,7 +27651,7 @@
         <v>2025</v>
       </c>
       <c r="E127">
-        <v>0.13153823842212123</v>
+        <v>0.868461761577879</v>
       </c>
       <c r="F127" t="b">
         <v>1</v>
@@ -27671,7 +27671,7 @@
         <v>2025</v>
       </c>
       <c r="E128">
-        <v>0.12960456347288019</v>
+        <v>0.87039543652712</v>
       </c>
       <c r="F128" t="b">
         <v>1</v>
@@ -27691,7 +27691,7 @@
         <v>2025</v>
       </c>
       <c r="E129">
-        <v>0.18853330755100067</v>
+        <v>0.811466692448999</v>
       </c>
       <c r="F129" t="b">
         <v>1</v>
@@ -27711,7 +27711,7 @@
         <v>2025</v>
       </c>
       <c r="E130">
-        <v>0.22570820845015951</v>
+        <v>0.774291791549841</v>
       </c>
       <c r="F130" t="b">
         <v>1</v>
@@ -27731,7 +27731,7 @@
         <v>2025</v>
       </c>
       <c r="E131">
-        <v>7.8603886686647959E-2</v>
+        <v>0.921396113313352</v>
       </c>
       <c r="F131" t="b">
         <v>1</v>
@@ -27751,7 +27751,7 @@
         <v>2025</v>
       </c>
       <c r="E132">
-        <v>0.16465242192787388</v>
+        <v>0.835347578072126</v>
       </c>
       <c r="F132" t="b">
         <v>1</v>
@@ -27771,7 +27771,7 @@
         <v>2025</v>
       </c>
       <c r="E133">
-        <v>0.11403848013148989</v>
+        <v>0.88596151986851</v>
       </c>
       <c r="F133" t="b">
         <v>1</v>
@@ -27791,7 +27791,7 @@
         <v>2025</v>
       </c>
       <c r="E134">
-        <v>8.6918688968384394E-2</v>
+        <v>0.913081311031616</v>
       </c>
       <c r="F134" t="b">
         <v>1</v>
@@ -27811,7 +27811,7 @@
         <v>2025</v>
       </c>
       <c r="E135">
-        <v>0.17997679590060908</v>
+        <v>0.820023204099391</v>
       </c>
       <c r="F135" t="b">
         <v>1</v>
@@ -27831,7 +27831,7 @@
         <v>2025</v>
       </c>
       <c r="E136">
-        <v>4.9598762448032484E-2</v>
+        <v>0.950401237551967</v>
       </c>
       <c r="F136" t="b">
         <v>1</v>
@@ -27851,7 +27851,7 @@
         <v>2025</v>
       </c>
       <c r="E137">
-        <v>9.755390118921009E-2</v>
+        <v>0.90244609881079</v>
       </c>
       <c r="F137" t="b">
         <v>1</v>
@@ -27871,7 +27871,7 @@
         <v>2025</v>
       </c>
       <c r="E138">
-        <v>0.10973605336942859</v>
+        <v>0.890263946630571</v>
       </c>
       <c r="F138" t="b">
         <v>1</v>
@@ -27891,7 +27891,7 @@
         <v>2025</v>
       </c>
       <c r="E139">
-        <v>7.8507202939185908E-2</v>
+        <v>0.921492797060814</v>
       </c>
       <c r="F139" t="b">
         <v>1</v>
@@ -27911,7 +27911,7 @@
         <v>2025</v>
       </c>
       <c r="E140">
-        <v>7.6235134873827701E-2</v>
+        <v>0.923764865126172</v>
       </c>
       <c r="F140" t="b">
         <v>1</v>
@@ -27931,7 +27931,7 @@
         <v>2025</v>
       </c>
       <c r="E141">
-        <v>0.11795417190370297</v>
+        <v>0.882045828096297</v>
       </c>
       <c r="F141" t="b">
         <v>1</v>
@@ -27951,7 +27951,7 @@
         <v>2025</v>
       </c>
       <c r="E142">
-        <v>0.15179348351542105</v>
+        <v>0.848206516484579</v>
       </c>
       <c r="F142" t="b">
         <v>1</v>
@@ -27971,7 +27971,7 @@
         <v>2025</v>
       </c>
       <c r="E143">
-        <v>0.14372039060233971</v>
+        <v>0.85627960939766</v>
       </c>
       <c r="F143" t="b">
         <v>1</v>
@@ -27991,7 +27991,7 @@
         <v>2025</v>
       </c>
       <c r="E144">
-        <v>5.9605530310354829E-2</v>
+        <v>0.940394469689645</v>
       </c>
       <c r="F144" t="b">
         <v>1</v>
@@ -28011,7 +28011,7 @@
         <v>2025</v>
       </c>
       <c r="E145">
-        <v>0.11311998453060039</v>
+        <v>0.8868800154694</v>
       </c>
       <c r="F145" t="b">
         <v>1</v>
@@ -28031,7 +28031,7 @@
         <v>2025</v>
       </c>
       <c r="E146">
-        <v>0.13236005027554867</v>
+        <v>0.867639949724451</v>
       </c>
       <c r="F146" t="b">
         <v>1</v>
@@ -28051,7 +28051,7 @@
         <v>2025</v>
       </c>
       <c r="E147">
-        <v>0.15585420090882723</v>
+        <v>0.844145799091173</v>
       </c>
       <c r="F147" t="b">
         <v>1</v>
@@ -28071,7 +28071,7 @@
         <v>2025</v>
       </c>
       <c r="E148">
-        <v>0.19017693125785554</v>
+        <v>0.809823068742144</v>
       </c>
       <c r="F148" t="b">
         <v>1</v>
@@ -28091,7 +28091,7 @@
         <v>2025</v>
       </c>
       <c r="E149">
-        <v>6.9032195687904863E-2</v>
+        <v>0.930967804312095</v>
       </c>
       <c r="F149" t="b">
         <v>1</v>
@@ -28111,7 +28111,7 @@
         <v>2025</v>
       </c>
       <c r="E150">
-        <v>0.48182345547713429</v>
+        <v>0.518176544522866</v>
       </c>
       <c r="F150" t="b">
         <v>1</v>
@@ -28131,7 +28131,7 @@
         <v>2025</v>
       </c>
       <c r="E151">
-        <v>0.14589577492023589</v>
+        <v>0.854104225079764</v>
       </c>
       <c r="F151" t="b">
         <v>1</v>
@@ -28151,7 +28151,7 @@
         <v>2025</v>
       </c>
       <c r="E152">
-        <v>0.12718746978632892</v>
+        <v>0.872812530213671</v>
       </c>
       <c r="F152" t="b">
         <v>1</v>
@@ -28171,7 +28171,7 @@
         <v>2025</v>
       </c>
       <c r="E153">
-        <v>5.2354249250700952E-2</v>
+        <v>0.947645750749299</v>
       </c>
       <c r="F153" t="b">
         <v>1</v>
@@ -28191,7 +28191,7 @@
         <v>2025</v>
       </c>
       <c r="E154">
-        <v>0.2019240065744948</v>
+        <v>0.798075993425505</v>
       </c>
       <c r="F154" t="b">
         <v>1</v>
@@ -28211,7 +28211,7 @@
         <v>2025</v>
       </c>
       <c r="E155">
-        <v>6.8983853814173837E-2</v>
+        <v>0.931016146185826</v>
       </c>
       <c r="F155" t="b">
         <v>1</v>
@@ -28231,7 +28231,7 @@
         <v>2025</v>
       </c>
       <c r="E156">
-        <v>0.11979116310548195</v>
+        <v>0.880208836894518</v>
       </c>
       <c r="F156" t="b">
         <v>1</v>
@@ -28251,7 +28251,7 @@
         <v>2025</v>
       </c>
       <c r="E157">
-        <v>0.12844435850333558</v>
+        <v>0.871555641496664</v>
       </c>
       <c r="F157" t="b">
         <v>1</v>
@@ -28271,7 +28271,7 @@
         <v>2025</v>
       </c>
       <c r="E158">
-        <v>0.20351928840761868</v>
+        <v>0.796480711592381</v>
       </c>
       <c r="F158" t="b">
         <v>1</v>
@@ -28291,7 +28291,7 @@
         <v>2025</v>
       </c>
       <c r="E159">
-        <v>6.9515614425215116E-2</v>
+        <v>0.930484385574785</v>
       </c>
       <c r="F159" t="b">
         <v>1</v>
@@ -28311,7 +28311,7 @@
         <v>2025</v>
       </c>
       <c r="E160">
-        <v>9.2091269457604152E-2</v>
+        <v>0.907908730542396</v>
       </c>
       <c r="F160" t="b">
         <v>1</v>
@@ -28331,7 +28331,7 @@
         <v>2025</v>
       </c>
       <c r="E161">
-        <v>6.6228367011505362E-2</v>
+        <v>0.933771632988495</v>
       </c>
       <c r="F161" t="b">
         <v>1</v>
@@ -28351,7 +28351,7 @@
         <v>2025</v>
       </c>
       <c r="E162">
-        <v>0.10175964420380931</v>
+        <v>0.898240355796191</v>
       </c>
       <c r="F162" t="b">
         <v>1</v>
@@ -28371,7 +28371,7 @@
         <v>2025</v>
       </c>
       <c r="E163">
-        <v>0.16909987431112827</v>
+        <v>0.830900125688872</v>
       </c>
       <c r="F163" t="b">
         <v>1</v>
@@ -28391,7 +28391,7 @@
         <v>2025</v>
       </c>
       <c r="E164">
-        <v>8.8078893937929018E-2</v>
+        <v>0.911921106062071</v>
       </c>
       <c r="F164" t="b">
         <v>1</v>
@@ -28411,7 +28411,7 @@
         <v>2025</v>
       </c>
       <c r="E165">
-        <v>0.11355506139417962</v>
+        <v>0.88644493860582</v>
       </c>
       <c r="F165" t="b">
         <v>1</v>
@@ -28431,7 +28431,7 @@
         <v>2025</v>
       </c>
       <c r="E166">
-        <v>6.7388571981049986E-2</v>
+        <v>0.93261142801895</v>
       </c>
       <c r="F166" t="b">
         <v>1</v>
@@ -28451,7 +28451,7 @@
         <v>2025</v>
       </c>
       <c r="E167">
-        <v>0.12037126559025427</v>
+        <v>0.879628734409746</v>
       </c>
       <c r="F167" t="b">
         <v>1</v>
@@ -28471,7 +28471,7 @@
         <v>2025</v>
       </c>
       <c r="E168">
-        <v>5.3031035482935321E-2</v>
+        <v>0.946968964517065</v>
       </c>
       <c r="F168" t="b">
         <v>1</v>
@@ -28491,7 +28491,7 @@
         <v>2025</v>
       </c>
       <c r="E169">
-        <v>0.2043411002610461</v>
+        <v>0.795658899738954</v>
       </c>
       <c r="F169" t="b">
         <v>1</v>
@@ -28511,7 +28511,7 @@
         <v>2025</v>
       </c>
       <c r="E170">
-        <v>7.207773373295949E-2</v>
+        <v>0.927922266267041</v>
       </c>
       <c r="F170" t="b">
         <v>1</v>
@@ -28531,7 +28531,7 @@
         <v>2025</v>
       </c>
       <c r="E171">
-        <v>9.4411679396693399E-2</v>
+        <v>0.905588320603307</v>
       </c>
       <c r="F171" t="b">
         <v>1</v>
@@ -28551,7 +28551,7 @@
         <v>2025</v>
       </c>
       <c r="E172">
-        <v>6.9080537561635888E-2</v>
+        <v>0.930919462438364</v>
       </c>
       <c r="F172" t="b">
         <v>1</v>
@@ -28571,7 +28571,7 @@
         <v>2025</v>
       </c>
       <c r="E173">
-        <v>0.1434786812336846</v>
+        <v>0.856521318766315</v>
       </c>
       <c r="F173" t="b">
         <v>1</v>
@@ -28591,7 +28591,7 @@
         <v>2025</v>
       </c>
       <c r="E174">
-        <v>0.1597698926810403</v>
+        <v>0.84023010731896</v>
       </c>
       <c r="F174" t="b">
         <v>1</v>
@@ -28611,7 +28611,7 @@
         <v>2025</v>
       </c>
       <c r="E175">
-        <v>0.25640529826936093</v>
+        <v>0.743594701730639</v>
       </c>
       <c r="F175" t="b">
         <v>1</v>
@@ -28631,7 +28631,7 @@
         <v>2025</v>
       </c>
       <c r="E176">
-        <v>0.12032292371652323</v>
+        <v>0.879677076283477</v>
       </c>
       <c r="F176" t="b">
         <v>1</v>
@@ -28651,7 +28651,7 @@
         <v>2025</v>
       </c>
       <c r="E177">
-        <v>0.13627574204776174</v>
+        <v>0.863724257952238</v>
       </c>
       <c r="F177" t="b">
         <v>1</v>
@@ -28671,7 +28671,7 @@
         <v>2025</v>
       </c>
       <c r="E178">
-        <v>1.8853330755100067E-2</v>
+        <v>0.9811466692449</v>
       </c>
       <c r="F178" t="b">
         <v>1</v>
@@ -28691,7 +28691,7 @@
         <v>2025</v>
       </c>
       <c r="E179">
-        <v>0.15556414966644105</v>
+        <v>0.844435850333559</v>
       </c>
       <c r="F179" t="b">
         <v>1</v>
@@ -28711,7 +28711,7 @@
         <v>2025</v>
       </c>
       <c r="E180">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F180" t="b">
         <v>1</v>
@@ -28731,7 +28731,7 @@
         <v>2025</v>
       </c>
       <c r="E181">
-        <v>0.14531567243546359</v>
+        <v>0.854684327564536</v>
       </c>
       <c r="F181" t="b">
         <v>1</v>
@@ -28751,7 +28751,7 @@
         <v>2025</v>
       </c>
       <c r="E182">
-        <v>0.26172290437977375</v>
+        <v>0.738277095620226</v>
       </c>
       <c r="F182" t="b">
         <v>1</v>
@@ -28771,7 +28771,7 @@
         <v>2025</v>
       </c>
       <c r="E183">
-        <v>0.18384414579909117</v>
+        <v>0.816155854200909</v>
       </c>
       <c r="F183" t="b">
         <v>1</v>
@@ -28791,7 +28791,7 @@
         <v>2025</v>
       </c>
       <c r="E184">
-        <v>7.9860775403654632E-2</v>
+        <v>0.920139224596345</v>
       </c>
       <c r="F184" t="b">
         <v>1</v>
@@ -28811,7 +28811,7 @@
         <v>2025</v>
       </c>
       <c r="E185">
-        <v>0.11476360823745527</v>
+        <v>0.885236391762545</v>
       </c>
       <c r="F185" t="b">
         <v>1</v>
@@ -28831,7 +28831,7 @@
         <v>2025</v>
       </c>
       <c r="E186">
-        <v>0.18766315382384219</v>
+        <v>0.812336846176158</v>
       </c>
       <c r="F186" t="b">
         <v>1</v>
@@ -28851,7 +28851,7 @@
         <v>2025</v>
       </c>
       <c r="E187">
-        <v>0.16392729382190852</v>
+        <v>0.836072706178091</v>
       </c>
       <c r="F187" t="b">
         <v>1</v>
@@ -28871,7 +28871,7 @@
         <v>2025</v>
       </c>
       <c r="E188">
-        <v>0.16658609687711495</v>
+        <v>0.833413903122885</v>
       </c>
       <c r="F188" t="b">
         <v>1</v>
@@ -28891,7 +28891,7 @@
         <v>2025</v>
       </c>
       <c r="E189">
-        <v>8.4453253408102086E-2</v>
+        <v>0.915546746591898</v>
       </c>
       <c r="F189" t="b">
         <v>1</v>
@@ -28911,7 +28911,7 @@
         <v>2025</v>
       </c>
       <c r="E190">
-        <v>0.20255245093299815</v>
+        <v>0.797447549067002</v>
       </c>
       <c r="F190" t="b">
         <v>1</v>
@@ -28931,7 +28931,7 @@
         <v>2025</v>
       </c>
       <c r="E191">
-        <v>0.222856037900029</v>
+        <v>0.777143962099971</v>
       </c>
       <c r="F191" t="b">
         <v>1</v>
@@ -28951,7 +28951,7 @@
         <v>2025</v>
       </c>
       <c r="E192">
-        <v>0.19530116987334428</v>
+        <v>0.804698830126656</v>
       </c>
       <c r="F192" t="b">
         <v>1</v>
@@ -28971,7 +28971,7 @@
         <v>2025</v>
       </c>
       <c r="E193">
-        <v>0.10011602049695444</v>
+        <v>0.899883979503046</v>
       </c>
       <c r="F193" t="b">
         <v>1</v>
@@ -28991,7 +28991,7 @@
         <v>2025</v>
       </c>
       <c r="E194">
-        <v>0.11234651455090398</v>
+        <v>0.887653485449096</v>
       </c>
       <c r="F194" t="b">
         <v>1</v>
@@ -29011,7 +29011,7 @@
         <v>2025</v>
       </c>
       <c r="E195">
-        <v>8.1842792226626701E-2</v>
+        <v>0.918157207773373</v>
       </c>
       <c r="F195" t="b">
         <v>1</v>
@@ -29031,7 +29031,7 @@
         <v>2025</v>
       </c>
       <c r="E196">
-        <v>0.56492313642076764</v>
+        <v>0.435076863579232</v>
       </c>
       <c r="F196" t="b">
         <v>1</v>
@@ -29051,7 +29051,7 @@
         <v>2025</v>
       </c>
       <c r="E197">
-        <v>5.254761674562506E-2</v>
+        <v>0.947452383254375</v>
       </c>
       <c r="F197" t="b">
         <v>1</v>
@@ -29071,7 +29071,7 @@
         <v>2025</v>
       </c>
       <c r="E198">
-        <v>7.8942279802765136E-2</v>
+        <v>0.921057720197235</v>
       </c>
       <c r="F198" t="b">
         <v>1</v>
@@ -29091,7 +29091,7 @@
         <v>2025</v>
       </c>
       <c r="E199">
-        <v>0.37083051339069906</v>
+        <v>0.629169486609301</v>
       </c>
       <c r="F199" t="b">
         <v>1</v>
@@ -29111,7 +29111,7 @@
         <v>2025</v>
       </c>
       <c r="E200">
-        <v>8.4356569660640035E-2</v>
+        <v>0.91564343033936</v>
       </c>
       <c r="F200" t="b">
         <v>1</v>
@@ -29131,7 +29131,7 @@
         <v>2025</v>
       </c>
       <c r="E201">
-        <v>8.8078893937929018E-2</v>
+        <v>0.911921106062071</v>
       </c>
       <c r="F201" t="b">
         <v>1</v>
@@ -29151,7 +29151,7 @@
         <v>2025</v>
       </c>
       <c r="E202">
-        <v>0.15928647394373002</v>
+        <v>0.84071352605627</v>
       </c>
       <c r="F202" t="b">
         <v>1</v>
@@ -29171,7 +29171,7 @@
         <v>2025</v>
       </c>
       <c r="E203">
-        <v>8.9045731412549539E-2</v>
+        <v>0.91095426858745</v>
       </c>
       <c r="F203" t="b">
         <v>1</v>
@@ -29191,7 +29191,7 @@
         <v>2025</v>
       </c>
       <c r="E204">
-        <v>0.11979116310548195</v>
+        <v>0.880208836894518</v>
       </c>
       <c r="F204" t="b">
         <v>1</v>
@@ -29211,7 +29211,7 @@
         <v>2025</v>
       </c>
       <c r="E205">
-        <v>9.5040123755196743E-2</v>
+        <v>0.904959876244803</v>
       </c>
       <c r="F205" t="b">
         <v>1</v>
@@ -29231,7 +29231,7 @@
         <v>2025</v>
       </c>
       <c r="E206">
-        <v>0.11133133520255244</v>
+        <v>0.888668664797448</v>
       </c>
       <c r="F206" t="b">
         <v>1</v>
@@ -29251,7 +29251,7 @@
         <v>2025</v>
       </c>
       <c r="E207">
-        <v>0.14473556995069126</v>
+        <v>0.855264430049309</v>
       </c>
       <c r="F207" t="b">
         <v>1</v>
@@ -29271,7 +29271,7 @@
         <v>2025</v>
       </c>
       <c r="E208">
-        <v>0.23619839504979212</v>
+        <v>0.763801604950208</v>
       </c>
       <c r="F208" t="b">
         <v>1</v>
@@ -29291,7 +29291,7 @@
         <v>2025</v>
       </c>
       <c r="E209">
-        <v>4.2492507009571689E-2</v>
+        <v>0.957507492990428</v>
       </c>
       <c r="F209" t="b">
         <v>1</v>
@@ -29311,7 +29311,7 @@
         <v>2025</v>
       </c>
       <c r="E210">
-        <v>0.3385864836121048</v>
+        <v>0.661413516387895</v>
       </c>
       <c r="F210" t="b">
         <v>1</v>
@@ -29331,7 +29331,7 @@
         <v>2025</v>
       </c>
       <c r="E211">
-        <v>5.878371845692739E-2</v>
+        <v>0.941216281543073</v>
       </c>
       <c r="F211" t="b">
         <v>1</v>
@@ -29351,7 +29351,7 @@
         <v>2025</v>
       </c>
       <c r="E212">
-        <v>0.21705501305230587</v>
+        <v>0.782944986947694</v>
       </c>
       <c r="F212" t="b">
         <v>1</v>
@@ -29371,7 +29371,7 @@
         <v>2025</v>
       </c>
       <c r="E213">
-        <v>0.1459441167939669</v>
+        <v>0.854055883206033</v>
       </c>
       <c r="F213" t="b">
         <v>1</v>
@@ -29391,7 +29391,7 @@
         <v>2025</v>
       </c>
       <c r="E214">
-        <v>6.2989461471526634E-2</v>
+        <v>0.937010538528473</v>
       </c>
       <c r="F214" t="b">
         <v>1</v>
@@ -29411,7 +29411,7 @@
         <v>2025</v>
       </c>
       <c r="E215">
-        <v>0.12017789809533017</v>
+        <v>0.87982210190467</v>
       </c>
       <c r="F215" t="b">
         <v>1</v>
@@ -29431,7 +29431,7 @@
         <v>2025</v>
       </c>
       <c r="E216">
-        <v>0.13245673402301072</v>
+        <v>0.867543265976989</v>
       </c>
       <c r="F216" t="b">
         <v>1</v>
@@ -29451,7 +29451,7 @@
         <v>2025</v>
       </c>
       <c r="E217">
-        <v>8.3099680943633361E-2</v>
+        <v>0.916900319056367</v>
       </c>
       <c r="F217" t="b">
         <v>1</v>
@@ -29471,7 +29471,7 @@
         <v>2025</v>
       </c>
       <c r="E218">
-        <v>0.21729672242096101</v>
+        <v>0.782703277579039</v>
       </c>
       <c r="F218" t="b">
         <v>1</v>
@@ -29491,7 +29491,7 @@
         <v>2025</v>
       </c>
       <c r="E219">
-        <v>7.6186793000096675E-2</v>
+        <v>0.923813206999903</v>
       </c>
       <c r="F219" t="b">
         <v>1</v>
@@ -29511,7 +29511,7 @@
         <v>2025</v>
       </c>
       <c r="E220">
-        <v>8.7015372715846459E-2</v>
+        <v>0.912984627284154</v>
       </c>
       <c r="F220" t="b">
         <v>1</v>

</xml_diff>